<commit_message>
Added comments to check_stock_alerts.py
</commit_message>
<xml_diff>
--- a/stocks.xlsx
+++ b/stocks.xlsx
@@ -1,35 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Suresh\PycharmProjects\scheduled-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71B67D93-8AB1-4050-8C91-2C8C97B6C73C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E283CAA-DAC5-45DE-96E5-106CCF38CA3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DBF5B9E9-41A4-47B0-865D-D7F003C09541}"/>
   </bookViews>
   <sheets>
     <sheet name="S Main" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
@@ -39,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="48">
   <si>
     <t>Name</t>
   </si>
@@ -180,6 +169,9 @@
   </si>
   <si>
     <t>YESBANK.BO</t>
+  </si>
+  <si>
+    <t>&gt;</t>
   </si>
 </sst>
 </file>
@@ -748,10 +740,14 @@
         <v>41</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
+        <v>41</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="4">
+        <v>25</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -824,10 +820,14 @@
         <v>41</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
+        <v>41</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G13" s="4">
+        <v>1000</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">

</xml_diff>

<commit_message>
Added Power Grid & REC Ltd
</commit_message>
<xml_diff>
--- a/stocks.xlsx
+++ b/stocks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Suresh\PycharmProjects\scheduled-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E283CAA-DAC5-45DE-96E5-106CCF38CA3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C366B789-049D-461A-9990-9A9F5B395186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DBF5B9E9-41A4-47B0-865D-D7F003C09541}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="53">
   <si>
     <t>Name</t>
   </si>
@@ -172,6 +172,21 @@
   </si>
   <si>
     <t>&gt;</t>
+  </si>
+  <si>
+    <t>&lt;</t>
+  </si>
+  <si>
+    <t>Power Grid</t>
+  </si>
+  <si>
+    <t>POWERGRID.BO</t>
+  </si>
+  <si>
+    <t>REC Ltd</t>
+  </si>
+  <si>
+    <t>RECLTD.BO</t>
   </si>
 </sst>
 </file>
@@ -247,7 +262,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -257,6 +272,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -562,7 +579,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FCA83A5-EE17-4E29-B37F-BCB7A5AAA969}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.88671875" bestFit="1" customWidth="1"/>
@@ -702,10 +719,14 @@
         <v>41</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
+        <v>41</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="4">
+        <v>260</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -801,10 +822,14 @@
         <v>41</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
+        <v>41</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" s="4">
+        <v>430</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
@@ -961,6 +986,52 @@
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" s="6">
+        <v>270</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G21" s="4">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" s="6">
+        <v>313</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G22" s="4">
+        <v>310</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added min, max & placement logic
</commit_message>
<xml_diff>
--- a/stocks.xlsx
+++ b/stocks.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Suresh\PycharmProjects\scheduled-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C366B789-049D-461A-9990-9A9F5B395186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEAA329B-3ACC-4A24-B280-BFD27B5F0E4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DBF5B9E9-41A4-47B0-865D-D7F003C09541}"/>
   </bookViews>
   <sheets>
     <sheet name="S Main" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'S Main'!$A$1:$G$22</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -262,7 +265,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -272,7 +275,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -621,7 +623,7 @@
         <v>172.81013157894733</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>42</v>
@@ -640,7 +642,7 @@
         <v>503.69607032558139</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>42</v>
@@ -659,7 +661,7 @@
         <v>57.830406026058633</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>42</v>
@@ -678,7 +680,7 @@
         <v>110.19422105670104</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>42</v>
@@ -697,7 +699,7 @@
         <v>554.99766666666665</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>42</v>
@@ -739,7 +741,7 @@
         <v>26.013505000000002</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>42</v>
@@ -781,7 +783,7 @@
         <v>23.33278516426159</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>42</v>
@@ -800,7 +802,7 @@
         <v>177.50579930069932</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>42</v>
@@ -865,7 +867,7 @@
         <v>119.79999999999998</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>42</v>
@@ -884,7 +886,7 @@
         <v>717.05555555555554</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>42</v>
@@ -903,7 +905,7 @@
         <v>44.493333333333332</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>42</v>
@@ -922,7 +924,7 @@
         <v>193</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>42</v>
@@ -941,7 +943,7 @@
         <v>155.83000000000001</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>42</v>
@@ -960,7 +962,7 @@
         <v>415</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>42</v>
@@ -979,7 +981,7 @@
         <v>2165</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>42</v>
@@ -988,13 +990,13 @@
       <c r="G20" s="4"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="5">
         <v>270</v>
       </c>
       <c r="D21" s="4" t="s">
@@ -1011,13 +1013,13 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="2" t="s">
         <v>51</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C22" s="6">
+      <c r="C22" s="5">
         <v>313</v>
       </c>
       <c r="D22" s="4" t="s">
@@ -1034,6 +1036,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G22" xr:uid="{8FCA83A5-EE17-4E29-B37F-BCB7A5AAA969}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>